<commit_message>
Actualização da pagina das Feiras
</commit_message>
<xml_diff>
--- a/BENEFICIARIOS_INDIRECTOS_Report.xlsx
+++ b/BENEFICIARIOS_INDIRECTOS_Report.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://muvamozorg.sharepoint.com/sites/mis.drive/Documentos Partilhados/PROJECTOS/Sistema de Monitoria/Abrindo_Oportunidades/2026/Dash_Abrindo_2026/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DionisioMahumane\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="11_4F6EF6C982138CB48E335FEBAA514FB25C7BA9D8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BAD511EA-5216-4301-A79C-BE5F645E514A}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E0908A7-CA97-45F4-88C5-B55ED968FC16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="90">
   <si>
     <t>Data de Registo</t>
   </si>
@@ -43,6 +43,69 @@
     <t>Monapo</t>
   </si>
   <si>
+    <t>Domingas Albino</t>
+  </si>
+  <si>
+    <t>MUTOCONE</t>
+  </si>
+  <si>
+    <t>ELSA ADAMUGE VASCO</t>
+  </si>
+  <si>
+    <t>Sim</t>
+  </si>
+  <si>
+    <t>Aina Vasco</t>
+  </si>
+  <si>
+    <t>Feminino</t>
+  </si>
+  <si>
+    <t>Membro da Família</t>
+  </si>
+  <si>
+    <t>Começou ajudar no negócio da família</t>
+  </si>
+  <si>
+    <t>Ajuda nas actividades de boa praticas Agrícolas</t>
+  </si>
+  <si>
+    <t>Não</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>+258871048164</t>
+  </si>
+  <si>
+    <t>PASCOELA DANIEL</t>
+  </si>
+  <si>
+    <t>Filomena Abacar</t>
+  </si>
+  <si>
+    <t>Venda de feijão fava</t>
+  </si>
+  <si>
+    <t>+258864152750</t>
+  </si>
+  <si>
+    <t>FILOMENA ALMEIDA</t>
+  </si>
+  <si>
+    <t>Alima Elias</t>
+  </si>
+  <si>
+    <t>Começou a trabalhar no negócio da família</t>
+  </si>
+  <si>
+    <t>Venda de farinha celeste</t>
+  </si>
+  <si>
+    <t>+258869636778</t>
+  </si>
+  <si>
     <t>Remigio Horacio</t>
   </si>
   <si>
@@ -52,15 +115,9 @@
     <t>ESMENIA HORLANDO</t>
   </si>
   <si>
-    <t>Sim</t>
-  </si>
-  <si>
     <t xml:space="preserve">Carla Inocêncio </t>
   </si>
   <si>
-    <t>Feminino</t>
-  </si>
-  <si>
     <t>Membro da comunidade</t>
   </si>
   <si>
@@ -70,9 +127,6 @@
     <t>Venda de bolinhos</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
     <t>+258874560080</t>
   </si>
   <si>
@@ -82,9 +136,6 @@
     <t>Masculino</t>
   </si>
   <si>
-    <t>Começou ajudar no negócio da família</t>
-  </si>
-  <si>
     <t>Venda de produtos agricolas</t>
   </si>
   <si>
@@ -100,9 +151,6 @@
     <t xml:space="preserve">Manuel Romeu Botão </t>
   </si>
   <si>
-    <t>Membro da Família</t>
-  </si>
-  <si>
     <t>Venda de galinha poedeira</t>
   </si>
   <si>
@@ -115,9 +163,6 @@
     <t>Vizinho</t>
   </si>
   <si>
-    <t>Começou a trabalhar no negócio da família</t>
-  </si>
-  <si>
     <t>Corte de arroz na machamba</t>
   </si>
   <si>
@@ -175,9 +220,6 @@
     <t>Debulha do milho</t>
   </si>
   <si>
-    <t>Não</t>
-  </si>
-  <si>
     <t>+258842395652</t>
   </si>
   <si>
@@ -211,12 +253,6 @@
     <t>+258868326323</t>
   </si>
   <si>
-    <t>Domingas Albino</t>
-  </si>
-  <si>
-    <t>MUTOCONE</t>
-  </si>
-  <si>
     <t>GUILHERMINA ABACAR</t>
   </si>
   <si>
@@ -229,6 +265,9 @@
     <t>+258863199673</t>
   </si>
   <si>
+    <t>Nome_Beneficiario_Indirecto</t>
+  </si>
+  <si>
     <t>Sexo</t>
   </si>
   <si>
@@ -247,13 +286,10 @@
     <t>Renda?</t>
   </si>
   <si>
+    <t>Contacto Proprio</t>
+  </si>
+  <si>
     <t>Contacto Alternativo</t>
-  </si>
-  <si>
-    <t>Contacto Proprio</t>
-  </si>
-  <si>
-    <t>Nome_Beneficiario_Indirecto</t>
   </si>
 </sst>
 </file>
@@ -630,7 +666,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O14"/>
+  <dimension ref="A1:O17"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelCol="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -661,36 +697,36 @@
         <v>5</v>
       </c>
       <c r="G1" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="H1" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="I1" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="J1" t="s">
-        <v>71</v>
+        <v>84</v>
       </c>
       <c r="K1" t="s">
-        <v>72</v>
+        <v>85</v>
       </c>
       <c r="L1" t="s">
-        <v>73</v>
+        <v>86</v>
       </c>
       <c r="M1" t="s">
-        <v>74</v>
+        <v>87</v>
       </c>
       <c r="N1" t="s">
-        <v>76</v>
+        <v>88</v>
       </c>
       <c r="O1" t="s">
-        <v>75</v>
+        <v>89</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
-        <v>46127</v>
+        <v>46203</v>
       </c>
       <c r="B2" t="s">
         <v>6</v>
@@ -714,7 +750,7 @@
         <v>12</v>
       </c>
       <c r="I2" s="2">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="J2" t="s">
         <v>13</v>
@@ -726,18 +762,18 @@
         <v>15</v>
       </c>
       <c r="M2" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="N2" t="s">
         <v>17</v>
       </c>
       <c r="O2" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
-        <v>46127</v>
+        <v>46203</v>
       </c>
       <c r="B3" t="s">
         <v>6</v>
@@ -749,25 +785,25 @@
         <v>8</v>
       </c>
       <c r="E3" t="s">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="F3" t="s">
         <v>10</v>
       </c>
       <c r="G3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H3" t="s">
+        <v>12</v>
+      </c>
+      <c r="I3" s="2">
         <v>19</v>
-      </c>
-      <c r="I3" s="2">
-        <v>23</v>
       </c>
       <c r="J3" t="s">
         <v>13</v>
       </c>
       <c r="K3" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="L3" t="s">
         <v>21</v>
@@ -776,212 +812,212 @@
         <v>10</v>
       </c>
       <c r="N3" t="s">
+        <v>17</v>
+      </c>
+      <c r="O3" t="s">
         <v>22</v>
-      </c>
-      <c r="O3" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
-        <v>46155</v>
+        <v>46203</v>
       </c>
       <c r="B4" t="s">
         <v>6</v>
       </c>
       <c r="C4" t="s">
-        <v>23</v>
+        <v>7</v>
       </c>
       <c r="D4" t="s">
         <v>8</v>
       </c>
       <c r="E4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" t="s">
+        <v>10</v>
+      </c>
+      <c r="G4" t="s">
         <v>24</v>
       </c>
-      <c r="F4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
+        <v>12</v>
+      </c>
+      <c r="I4" s="2">
+        <v>30</v>
+      </c>
+      <c r="J4" t="s">
+        <v>13</v>
+      </c>
+      <c r="K4" t="s">
         <v>25</v>
       </c>
-      <c r="H4" t="s">
-        <v>19</v>
-      </c>
-      <c r="I4" s="2">
-        <v>23</v>
-      </c>
-      <c r="J4" t="s">
+      <c r="L4" t="s">
         <v>26</v>
       </c>
-      <c r="K4" t="s">
-        <v>14</v>
-      </c>
-      <c r="L4" t="s">
+      <c r="M4" t="s">
+        <v>10</v>
+      </c>
+      <c r="N4" t="s">
+        <v>17</v>
+      </c>
+      <c r="O4" t="s">
         <v>27</v>
-      </c>
-      <c r="M4" t="s">
-        <v>10</v>
-      </c>
-      <c r="N4" t="s">
-        <v>28</v>
-      </c>
-      <c r="O4" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
-        <v>46155</v>
+        <v>46127</v>
       </c>
       <c r="B5" t="s">
         <v>6</v>
       </c>
       <c r="C5" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="D5" t="s">
-        <v>8</v>
+        <v>29</v>
       </c>
       <c r="E5" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="F5" t="s">
         <v>10</v>
       </c>
       <c r="G5" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="H5" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="I5" s="2">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="J5" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="K5" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="L5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="M5" t="s">
         <v>10</v>
       </c>
       <c r="N5" t="s">
-        <v>33</v>
+        <v>17</v>
       </c>
       <c r="O5" t="s">
-        <v>16</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
-        <v>46153</v>
+        <v>46127</v>
       </c>
       <c r="B6" t="s">
         <v>6</v>
       </c>
       <c r="C6" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" t="s">
+        <v>29</v>
+      </c>
+      <c r="E6" t="s">
+        <v>30</v>
+      </c>
+      <c r="F6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G6" t="s">
+        <v>36</v>
+      </c>
+      <c r="H6" t="s">
+        <v>37</v>
+      </c>
+      <c r="I6" s="2">
         <v>23</v>
       </c>
-      <c r="D6" t="s">
-        <v>8</v>
-      </c>
-      <c r="E6" t="s">
-        <v>34</v>
-      </c>
-      <c r="F6" t="s">
-        <v>10</v>
-      </c>
-      <c r="G6" t="s">
-        <v>35</v>
-      </c>
-      <c r="H6" t="s">
-        <v>12</v>
-      </c>
-      <c r="I6" s="2">
-        <v>26</v>
-      </c>
       <c r="J6" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="K6" t="s">
         <v>14</v>
       </c>
       <c r="L6" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="M6" t="s">
         <v>10</v>
       </c>
       <c r="N6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="O6" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
-        <v>46153</v>
+        <v>46155</v>
       </c>
       <c r="B7" t="s">
         <v>6</v>
       </c>
       <c r="C7" t="s">
+        <v>40</v>
+      </c>
+      <c r="D7" t="s">
+        <v>29</v>
+      </c>
+      <c r="E7" t="s">
+        <v>41</v>
+      </c>
+      <c r="F7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G7" t="s">
+        <v>42</v>
+      </c>
+      <c r="H7" t="s">
+        <v>37</v>
+      </c>
+      <c r="I7" s="2">
         <v>23</v>
       </c>
-      <c r="D7" t="s">
-        <v>8</v>
-      </c>
-      <c r="E7" t="s">
-        <v>34</v>
-      </c>
-      <c r="F7" t="s">
-        <v>10</v>
-      </c>
-      <c r="G7" t="s">
-        <v>38</v>
-      </c>
-      <c r="H7" t="s">
-        <v>12</v>
-      </c>
-      <c r="I7" s="2">
-        <v>20</v>
-      </c>
       <c r="J7" t="s">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="K7" t="s">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="L7" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="M7" t="s">
         <v>10</v>
       </c>
       <c r="N7" t="s">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="O7" t="s">
-        <v>16</v>
+        <v>44</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
-        <v>46153</v>
+        <v>46155</v>
       </c>
       <c r="B8" t="s">
         <v>6</v>
       </c>
       <c r="C8" t="s">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="D8" t="s">
-        <v>8</v>
+        <v>29</v>
       </c>
       <c r="E8" t="s">
         <v>41</v>
@@ -990,31 +1026,31 @@
         <v>10</v>
       </c>
       <c r="G8" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="H8" t="s">
-        <v>12</v>
+        <v>37</v>
       </c>
       <c r="I8" s="2">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="J8" t="s">
-        <v>13</v>
+        <v>46</v>
       </c>
       <c r="K8" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="L8" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="M8" t="s">
         <v>10</v>
       </c>
       <c r="N8" t="s">
-        <v>44</v>
+        <v>17</v>
       </c>
       <c r="O8" t="s">
-        <v>16</v>
+        <v>48</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
@@ -1025,151 +1061,151 @@
         <v>6</v>
       </c>
       <c r="C9" t="s">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="D9" t="s">
-        <v>8</v>
+        <v>29</v>
       </c>
       <c r="E9" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="F9" t="s">
         <v>10</v>
       </c>
       <c r="G9" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="H9" t="s">
         <v>12</v>
       </c>
       <c r="I9" s="2">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="J9" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="K9" t="s">
-        <v>14</v>
+        <v>33</v>
       </c>
       <c r="L9" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="M9" t="s">
         <v>10</v>
       </c>
       <c r="N9" t="s">
-        <v>16</v>
+        <v>52</v>
       </c>
       <c r="O9" t="s">
-        <v>47</v>
+        <v>17</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
-        <v>46150</v>
+        <v>46153</v>
       </c>
       <c r="B10" t="s">
         <v>6</v>
       </c>
       <c r="C10" t="s">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="D10" t="s">
-        <v>8</v>
+        <v>29</v>
       </c>
       <c r="E10" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F10" t="s">
         <v>10</v>
       </c>
       <c r="G10" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="H10" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="I10" s="2">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J10" t="s">
-        <v>30</v>
+        <v>46</v>
       </c>
       <c r="K10" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="L10" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="M10" t="s">
-        <v>51</v>
+        <v>10</v>
       </c>
       <c r="N10" t="s">
-        <v>52</v>
+        <v>17</v>
       </c>
       <c r="O10" t="s">
-        <v>16</v>
+        <v>55</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
-        <v>46150</v>
+        <v>46153</v>
       </c>
       <c r="B11" t="s">
         <v>6</v>
       </c>
       <c r="C11" t="s">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="D11" t="s">
-        <v>8</v>
+        <v>29</v>
       </c>
       <c r="E11" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="F11" t="s">
         <v>10</v>
       </c>
       <c r="G11" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="H11" t="s">
         <v>12</v>
       </c>
       <c r="I11" s="2">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="J11" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="K11" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="L11" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="M11" t="s">
         <v>10</v>
       </c>
       <c r="N11" t="s">
-        <v>55</v>
+        <v>17</v>
       </c>
       <c r="O11" t="s">
-        <v>16</v>
+        <v>59</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
-        <v>46148</v>
+        <v>46153</v>
       </c>
       <c r="B12" t="s">
         <v>6</v>
       </c>
       <c r="C12" t="s">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="D12" t="s">
-        <v>8</v>
+        <v>29</v>
       </c>
       <c r="E12" t="s">
         <v>56</v>
@@ -1178,125 +1214,266 @@
         <v>10</v>
       </c>
       <c r="G12" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="H12" t="s">
         <v>12</v>
       </c>
       <c r="I12" s="2">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="J12" t="s">
         <v>13</v>
       </c>
       <c r="K12" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="L12" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="M12" t="s">
         <v>10</v>
       </c>
       <c r="N12" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="O12" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
-        <v>46148</v>
+        <v>46150</v>
       </c>
       <c r="B13" t="s">
         <v>6</v>
       </c>
       <c r="C13" t="s">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="D13" t="s">
-        <v>8</v>
+        <v>29</v>
       </c>
       <c r="E13" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="F13" t="s">
         <v>10</v>
       </c>
       <c r="G13" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="H13" t="s">
+        <v>37</v>
+      </c>
+      <c r="I13" s="2">
         <v>19</v>
       </c>
-      <c r="I13" s="2">
-        <v>20</v>
-      </c>
       <c r="J13" t="s">
-        <v>26</v>
+        <v>46</v>
       </c>
       <c r="K13" t="s">
         <v>14</v>
       </c>
       <c r="L13" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="M13" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="N13" t="s">
-        <v>62</v>
+        <v>17</v>
       </c>
       <c r="O13" t="s">
-        <v>16</v>
+        <v>66</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
-        <v>46171</v>
+        <v>46150</v>
       </c>
       <c r="B14" t="s">
         <v>6</v>
       </c>
       <c r="C14" t="s">
+        <v>40</v>
+      </c>
+      <c r="D14" t="s">
+        <v>29</v>
+      </c>
+      <c r="E14" t="s">
         <v>63</v>
       </c>
-      <c r="D14" t="s">
-        <v>64</v>
-      </c>
-      <c r="E14" t="s">
-        <v>65</v>
-      </c>
       <c r="F14" t="s">
         <v>10</v>
       </c>
       <c r="G14" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H14" t="s">
         <v>12</v>
       </c>
       <c r="I14" s="2">
+        <v>28</v>
+      </c>
+      <c r="J14" t="s">
+        <v>13</v>
+      </c>
+      <c r="K14" t="s">
+        <v>33</v>
+      </c>
+      <c r="L14" t="s">
+        <v>68</v>
+      </c>
+      <c r="M14" t="s">
+        <v>10</v>
+      </c>
+      <c r="N14" t="s">
+        <v>17</v>
+      </c>
+      <c r="O14" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A15" s="1">
+        <v>46148</v>
+      </c>
+      <c r="B15" t="s">
+        <v>6</v>
+      </c>
+      <c r="C15" t="s">
+        <v>40</v>
+      </c>
+      <c r="D15" t="s">
+        <v>29</v>
+      </c>
+      <c r="E15" t="s">
+        <v>70</v>
+      </c>
+      <c r="F15" t="s">
+        <v>10</v>
+      </c>
+      <c r="G15" t="s">
+        <v>71</v>
+      </c>
+      <c r="H15" t="s">
+        <v>12</v>
+      </c>
+      <c r="I15" s="2">
+        <v>19</v>
+      </c>
+      <c r="J15" t="s">
+        <v>32</v>
+      </c>
+      <c r="K15" t="s">
+        <v>25</v>
+      </c>
+      <c r="L15" t="s">
+        <v>72</v>
+      </c>
+      <c r="M15" t="s">
+        <v>10</v>
+      </c>
+      <c r="N15" t="s">
+        <v>17</v>
+      </c>
+      <c r="O15" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A16" s="1">
+        <v>46148</v>
+      </c>
+      <c r="B16" t="s">
+        <v>6</v>
+      </c>
+      <c r="C16" t="s">
+        <v>40</v>
+      </c>
+      <c r="D16" t="s">
+        <v>29</v>
+      </c>
+      <c r="E16" t="s">
+        <v>70</v>
+      </c>
+      <c r="F16" t="s">
+        <v>10</v>
+      </c>
+      <c r="G16" t="s">
+        <v>74</v>
+      </c>
+      <c r="H16" t="s">
+        <v>37</v>
+      </c>
+      <c r="I16" s="2">
+        <v>20</v>
+      </c>
+      <c r="J16" t="s">
+        <v>13</v>
+      </c>
+      <c r="K16" t="s">
+        <v>33</v>
+      </c>
+      <c r="L16" t="s">
+        <v>75</v>
+      </c>
+      <c r="M16" t="s">
+        <v>10</v>
+      </c>
+      <c r="N16" t="s">
+        <v>17</v>
+      </c>
+      <c r="O16" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A17" s="1">
+        <v>46171</v>
+      </c>
+      <c r="B17" t="s">
+        <v>6</v>
+      </c>
+      <c r="C17" t="s">
+        <v>7</v>
+      </c>
+      <c r="D17" t="s">
+        <v>8</v>
+      </c>
+      <c r="E17" t="s">
+        <v>77</v>
+      </c>
+      <c r="F17" t="s">
+        <v>10</v>
+      </c>
+      <c r="G17" t="s">
+        <v>78</v>
+      </c>
+      <c r="H17" t="s">
+        <v>12</v>
+      </c>
+      <c r="I17" s="2">
         <v>9</v>
       </c>
-      <c r="J14" t="s">
-        <v>26</v>
-      </c>
-      <c r="K14" t="s">
-        <v>20</v>
-      </c>
-      <c r="L14" t="s">
-        <v>67</v>
-      </c>
-      <c r="M14" t="s">
-        <v>10</v>
-      </c>
-      <c r="N14" t="s">
-        <v>16</v>
-      </c>
-      <c r="O14" t="s">
-        <v>68</v>
+      <c r="J17" t="s">
+        <v>13</v>
+      </c>
+      <c r="K17" t="s">
+        <v>14</v>
+      </c>
+      <c r="L17" t="s">
+        <v>79</v>
+      </c>
+      <c r="M17" t="s">
+        <v>10</v>
+      </c>
+      <c r="N17" t="s">
+        <v>80</v>
+      </c>
+      <c r="O17" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -1305,28 +1482,8 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="54c5ab46-7543-4aba-b0fa-79d6a199bef5" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="20d57abc-823c-4051-a81a-1a0a01a8f39e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100DC8BB5B596CFDD4794B3344F0E8F53A4" ma:contentTypeVersion="15" ma:contentTypeDescription="Criar um novo documento." ma:contentTypeScope="" ma:versionID="9a7078cd21229583650f2264465a1c40">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="20d57abc-823c-4051-a81a-1a0a01a8f39e" xmlns:ns3="54c5ab46-7543-4aba-b0fa-79d6a199bef5" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4e45437c47114f519c494620e3e4bb67" ns2:_="" ns3:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100DC8BB5B596CFDD4794B3344F0E8F53A4" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="481cb719fb2f51215cc00c8d40533043">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="20d57abc-823c-4051-a81a-1a0a01a8f39e" xmlns:ns3="54c5ab46-7543-4aba-b0fa-79d6a199bef5" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="71df0815368817fe9627576b1e062219" ns2:_="" ns3:_="">
     <xsd:import namespace="20d57abc-823c-4051-a81a-1a0a01a8f39e"/>
     <xsd:import namespace="54c5ab46-7543-4aba-b0fa-79d6a199bef5"/>
     <xsd:element name="properties">
@@ -1399,7 +1556,7 @@
         <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Etiquetas de Imagem" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="edc6e55a-975c-4e83-894d-449406ca2714" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="edc6e55a-975c-4e83-894d-449406ca2714" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
       <xsd:complexType>
         <xsd:sequence>
           <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
@@ -1422,7 +1579,7 @@
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="54c5ab46-7543-4aba-b0fa-79d6a199bef5" elementFormDefault="qualified">
     <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="SharedWithUsers" ma:index="12" nillable="true" ma:displayName="Partilhado Com" ma:internalName="SharedWithUsers" ma:readOnly="true">
+    <xsd:element name="SharedWithUsers" ma:index="12" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
       <xsd:complexType>
         <xsd:complexContent>
           <xsd:extension base="dms:UserMulti">
@@ -1441,7 +1598,7 @@
         </xsd:complexContent>
       </xsd:complexType>
     </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="13" nillable="true" ma:displayName="Detalhes de Partilhado Com" ma:internalName="SharedWithDetails" ma:readOnly="true">
+    <xsd:element name="SharedWithDetails" ma:index="13" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Note">
           <xsd:maxLength value="255"/>
@@ -1469,8 +1626,8 @@
         <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo de Conteúdo"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Título"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
         <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
         <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
@@ -1559,40 +1716,34 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="20d57abc-823c-4051-a81a-1a0a01a8f39e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="54c5ab46-7543-4aba-b0fa-79d6a199bef5" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E1106C8C-38B7-458D-8D6D-DEADA3AB6F35}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EC9F28E0-0753-4232-B595-9195CFE227A4}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{91707975-E089-44C6-9E4C-BFEF0CB5B42A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="54c5ab46-7543-4aba-b0fa-79d6a199bef5"/>
-    <ds:schemaRef ds:uri="20d57abc-823c-4051-a81a-1a0a01a8f39e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{41296AD5-6CC4-466F-82EE-05D4A63C33AE}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B9FC7767-B7B5-4BEC-841D-E7073AC4EB6D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="20d57abc-823c-4051-a81a-1a0a01a8f39e"/>
-    <ds:schemaRef ds:uri="54c5ab46-7543-4aba-b0fa-79d6a199bef5"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{47E79391-6407-40CC-BCE2-5F9C11BAC4E3}"/>
 </file>
</xml_diff>